<commit_message>
Update Parent/Guardian Notification email template (ET-002)
- New subject: Incident Involving Your Child - {{incident_type}} - {{incident_id}}
- Body opens with "Hello," and uses literal INSERT NAME / PHONE# / EMAIL
  placeholders for the contact line
- Drop unused variables: parent_name, contact_name, contact_phone, contact_email
- Regenerate Incident-Tracker-Seed-Catalog.xlsx to stay in sync

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Incident-Tracker-Seed-Catalog.xlsx
+++ b/Incident-Tracker-Seed-Catalog.xlsx
@@ -3723,12 +3723,12 @@
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>[Incident Tracker] Bus Incident Involving Your Child - {{incident_id}}</t>
+          <t>Incident Involving Your Child - {{incident_type}} - {{incident_id}}</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>Dear {{parent_name}},
+          <t>Hello,
 We are writing to inform you of an incident that occurred on {{incident_date}} involving your child, {{student_name}}, while riding {{bus_route}}.
 Incident Type: {{incident_type}}
 Severity: {{severity}}
@@ -3737,7 +3737,7 @@
 {{incident_summary}}
 Immediate actions taken:
 {{actions_taken}}
-If you have any questions or concerns, please contact {{contact_name}} at {{contact_phone}} or {{contact_email}}.
+If you have any questions or concerns, please contact INSERT NAME at PHONE# or EMAIL.
 Sincerely,
 {{sender_name}}
 {{sender_title}}
@@ -3746,7 +3746,7 @@
       </c>
       <c r="H3" s="8" t="inlineStr">
         <is>
-          <t>parent_name, student_name, bus_route, incident_date, incident_type, severity, incident_location, incident_summary, actions_taken, contact_name, contact_phone, contact_email, sender_name, sender_title</t>
+          <t>student_name, bus_route, incident_date, incident_type, severity, incident_location, incident_summary, actions_taken, sender_name, sender_title</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Generalize Urgent Action Required -> Action Required email template
- Rename ET to "Action Required" and remove urgent-only language so it
  applies to routine and time-sensitive steps alike
- New subject "Action Required: {{step_name}} - {{incident_id}}"; body opens
  with "Hello," (drop recipient_name var)
- Renumber template IDs alphabetically per convention: Action Required=ET-001,
  Approval Request=ET-002, Parent/Guardian Notification=ET-003
- Regenerate Incident-Tracker-Seed-Catalog.xlsx to stay in sync

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Incident-Tracker-Seed-Catalog.xlsx
+++ b/Incident-Tracker-Seed-Catalog.xlsx
@@ -3651,30 +3651,80 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
+          <t>Action Required</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Notification</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>General notification that a workflow step requires action by the assigned role. Suitable for routine and time-sensitive steps alike.</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Action Required: {{step_name}} - {{incident_id}}</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Hello,
+A workflow step requires your attention:
+Step: {{step_name}}
+Incident: {{incident_id}}
+Severity: {{severity}}
+Assigned To: {{assigned_role}}
+Please log in to the Incident Tracker to review and complete this step.
+Thank you,
+Incident Tracker System</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>step_name, incident_id, severity, assigned_role</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>ET-002</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
           <t>Approval Request</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Approval</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>Sent to designated approvers when a step requires approval before proceeding.</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr">
         <is>
           <t>Approval needed for workflow step: {{step_name}} ({{incident_id}})</t>
         </is>
       </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>Hello,
 Your approval is needed for the following workflow step:
@@ -3689,44 +3739,44 @@
 Incident Tracker System</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="H3" s="8" t="inlineStr">
         <is>
           <t>step_name, incident_id, requested_by, request_date, step_description</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>ET-002</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>ET-003</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Parent/Guardian Notification</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Notification</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>Sent to parents or guardians when their child is involved in a bus incident. Used across most student-related workflows.</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Incident Involving Your Child - {{incident_type}} - {{incident_id}}</t>
         </is>
       </c>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>Hello,
 We are writing to inform you of an incident that occurred on {{incident_date}} involving your child, {{student_name}}, while riding {{bus_route}}.
@@ -3744,61 +3794,9 @@
 Student Transportation Department</t>
         </is>
       </c>
-      <c r="H3" s="8" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>student_name, bus_route, incident_date, incident_type, severity, incident_location, incident_summary, actions_taken, sender_name, sender_title</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>ET-003</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Urgent Action Required</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Notification</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>High-priority notification for critical or time-sensitive workflow steps.</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>[URGENT] Action Required: {{step_name}} - {{incident_id}}</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>URGENT: Immediate action is required.
-Hello {{recipient_name}},
-A high-priority workflow step requires your immediate attention:
-Step: {{step_name}}
-Incident: {{incident_id}}
-Severity: {{severity}}
-Assigned To: {{assigned_role}}
-Please log in to the Incident Tracker immediately to address this matter.
-This notification was sent because the incident severity is {{severity}} and requires prompt resolution.
-Thank you,
-Incident Tracker System</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>recipient_name, step_name, incident_id, severity, assigned_role</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Physical Altercation step 2: reframe as tablet-app incident submission
The driver notifies the safety coordinator by submitting the incident in the
tablet app, so rename "Safety Coordinator Notification" to "Submit Incident
Report via Tablet App" and describe submitting details (what occurred,
injuries, threatening behavior) via the app, which notifies the coordinator.
Regenerated Incident-Tracker-Seed-Catalog.xlsx to match.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Incident-Tracker-Seed-Catalog.xlsx
+++ b/Incident-Tracker-Seed-Catalog.xlsx
@@ -1563,12 +1563,12 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Safety Coordinator Notification</t>
+          <t>Submit Incident Report via Tablet App</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Notify safety coordinator of incident details, injuries, and any threatening behavior</t>
+          <t>Driver submits the incident details — what occurred, injuries, and any threatening behavior — through the tablet app. Submitting the report notifies the safety coordinator.</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Physical Altercation step 2: rename to "Submit Incident Report", drop email
Shorten the step name to "Submit Incident Report" and remove its email
notification config (no email on this step). Updated workflows.ts and the
generator; regenerated Incident-Tracker-Seed-Catalog.xlsx to match.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Incident-Tracker-Seed-Catalog.xlsx
+++ b/Incident-Tracker-Seed-Catalog.xlsx
@@ -1563,7 +1563,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Submit Incident Report via Tablet App</t>
+          <t>Submit Incident Report</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -1601,26 +1601,10 @@
       <c r="M6" s="5" t="inlineStr"/>
       <c r="N6" s="5" t="inlineStr"/>
       <c r="O6" s="5" t="inlineStr"/>
-      <c r="P6" s="5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="Q6" s="5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="R6" s="5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="S6" s="5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
+      <c r="P6" s="5" t="inlineStr"/>
+      <c r="Q6" s="5" t="inlineStr"/>
+      <c r="R6" s="5" t="inlineStr"/>
+      <c r="S6" s="5" t="inlineStr"/>
       <c r="T6" s="5" t="inlineStr"/>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Physical Altercation step 3: send Parent Notification email after the step
Change the Parent Notification email to fire on step completion instead of on
start (notifyOnStart false, notifyOnComplete true). Updated workflows.ts and
the generator; regenerated Incident-Tracker-Seed-Catalog.xlsx to match.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Incident-Tracker-Seed-Catalog.xlsx
+++ b/Incident-Tracker-Seed-Catalog.xlsx
@@ -1663,12 +1663,12 @@
       <c r="O7" s="7" t="inlineStr"/>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="R7" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Physical Altercation step 4: send Action Required to Safety Coordinator after step
Disciplinary Action Review now sends the "Action Required" email template to the
Safety Coordinator role, after the step completes (notifyOnStart false,
notifyOnComplete true; notifyGroups: Safety Coordinator; emailTemplate: Action
Required). UI reflects this via existing template/timing/notify-roles controls.

Seed catalog: add a notify_groups column to the Workflow Steps sheet and refresh
README notes (a step now references a template; document notify_groups + timing).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Incident-Tracker-Seed-Catalog.xlsx
+++ b/Incident-Tracker-Seed-Catalog.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Incident Types'!$A$1:$F$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Workflows'!$A$1:$E$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Workflow Steps'!$A$1:$T$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Workflow Steps'!$A$1:$U$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Step Templates'!$A$1:$K$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Email Templates'!$A$1:$H$4</definedName>
   </definedNames>
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B30"/>
+  <dimension ref="B1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -646,50 +646,57 @@
     <row r="23">
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>• 'email_template' on a step references Email Templates.name. A blank means the step sends no templated email (though notify_* flags may still be set). In the current configuration no step references a template, but the templates remain seeded as a reusable library.</t>
+          <t>• 'email_template' on a step references Email Templates.name. A blank means the step sends no templated email (though notify_* flags may still be set). Currently only WF-002 step 4 references a template ('Action Required'); the others are seeded as a reusable library.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>• Every workflow step is manually triggered (trigger_type = manual); there are no time-delay/conditional/auto-advance steps in the current configuration.</t>
+          <t>• 'notify_groups' lists the roles that should receive the step's email (comma-separated). 'notify_on_start' / 'notify_on_complete' indicate timing: notify before the step starts vs. after it completes.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>• estimated_duration / default_duration are free-text labels ('15 minutes', '2 hours'); keep as text unless you parse them into minutes.</t>
+          <t>• Every workflow step is manually triggered (trigger_type = manual); there are no time-delay/conditional/auto-advance steps in the current configuration.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>• Email template variables are listed without the surrounding {{ }} braces; the body shows the {{placeholder}} form.</t>
+          <t>• estimated_duration / default_duration are free-text labels ('15 minutes', '2 hours'); keep as text unless you parse them into minutes.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>• 'Witness / Bystander Statement' (incident type + WF-006) is intentionally non-disciplinary: no parent notification or approval steps, so a student who only witnessed/helped is not flagged on a disciplinary incident.</t>
+          <t>• Email template variables are listed without the surrounding {{ }} braces; the body shows the {{placeholder}} form.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="2" t="inlineStr">
         <is>
+          <t>• 'Witness / Bystander Statement' (incident type + WF-006) is intentionally non-disciplinary: no parent notification or approval steps, so a student who only witnessed/helped is not flagged on a disciplinary incident.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="2" t="inlineStr">
+        <is>
           <t>• Severity values: Low, Medium, High, Critical.   applicable_to values: student, driver, both.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="B29" s="2" t="inlineStr"/>
-    </row>
     <row r="30">
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>Generated by gen_seed_catalog_xlsx.py — re-run after editing the app data files to refresh.</t>
         </is>
@@ -1164,7 +1171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T27"/>
+  <dimension ref="A1:U27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1186,7 +1193,8 @@
     <col width="15" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="26" customWidth="1" min="20" max="20"/>
+    <col width="22" customWidth="1" min="20" max="20"/>
+    <col width="26" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1286,6 +1294,11 @@
         </is>
       </c>
       <c r="T1" s="4" t="inlineStr">
+        <is>
+          <t>notify_groups</t>
+        </is>
+      </c>
+      <c r="U1" s="4" t="inlineStr">
         <is>
           <t>additional_recipients</t>
         </is>
@@ -1350,6 +1363,7 @@
       <c r="R2" s="5" t="inlineStr"/>
       <c r="S2" s="5" t="inlineStr"/>
       <c r="T2" s="5" t="inlineStr"/>
+      <c r="U2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -1426,6 +1440,7 @@
         </is>
       </c>
       <c r="T3" s="7" t="inlineStr"/>
+      <c r="U3" s="7" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -1486,6 +1501,7 @@
       <c r="R4" s="5" t="inlineStr"/>
       <c r="S4" s="5" t="inlineStr"/>
       <c r="T4" s="5" t="inlineStr"/>
+      <c r="U4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -1546,6 +1562,7 @@
       <c r="R5" s="7" t="inlineStr"/>
       <c r="S5" s="7" t="inlineStr"/>
       <c r="T5" s="7" t="inlineStr"/>
+      <c r="U5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -1606,6 +1623,7 @@
       <c r="R6" s="5" t="inlineStr"/>
       <c r="S6" s="5" t="inlineStr"/>
       <c r="T6" s="5" t="inlineStr"/>
+      <c r="U6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -1682,6 +1700,7 @@
         </is>
       </c>
       <c r="T7" s="7" t="inlineStr"/>
+      <c r="U7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -1740,10 +1759,14 @@
       <c r="L8" s="5" t="inlineStr"/>
       <c r="M8" s="5" t="inlineStr"/>
       <c r="N8" s="5" t="inlineStr"/>
-      <c r="O8" s="5" t="inlineStr"/>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Action Required</t>
+        </is>
+      </c>
       <c r="P8" s="5" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="Q8" s="5" t="inlineStr">
@@ -1761,7 +1784,12 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="T8" s="5" t="inlineStr"/>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>Safety Coordinator</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -1822,6 +1850,7 @@
       <c r="R9" s="7" t="inlineStr"/>
       <c r="S9" s="7" t="inlineStr"/>
       <c r="T9" s="7" t="inlineStr"/>
+      <c r="U9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -1882,6 +1911,7 @@
       <c r="R10" s="5" t="inlineStr"/>
       <c r="S10" s="5" t="inlineStr"/>
       <c r="T10" s="5" t="inlineStr"/>
+      <c r="U10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -1958,6 +1988,7 @@
         </is>
       </c>
       <c r="T11" s="7" t="inlineStr"/>
+      <c r="U11" s="7" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -2034,6 +2065,7 @@
         </is>
       </c>
       <c r="T12" s="5" t="inlineStr"/>
+      <c r="U12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -2114,6 +2146,7 @@
         </is>
       </c>
       <c r="T13" s="7" t="inlineStr"/>
+      <c r="U13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -2174,6 +2207,7 @@
       <c r="R14" s="5" t="inlineStr"/>
       <c r="S14" s="5" t="inlineStr"/>
       <c r="T14" s="5" t="inlineStr"/>
+      <c r="U14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -2234,6 +2268,7 @@
       <c r="R15" s="7" t="inlineStr"/>
       <c r="S15" s="7" t="inlineStr"/>
       <c r="T15" s="7" t="inlineStr"/>
+      <c r="U15" s="7" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -2310,6 +2345,7 @@
         </is>
       </c>
       <c r="T16" s="5" t="inlineStr"/>
+      <c r="U16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -2370,6 +2406,7 @@
       <c r="R17" s="7" t="inlineStr"/>
       <c r="S17" s="7" t="inlineStr"/>
       <c r="T17" s="7" t="inlineStr"/>
+      <c r="U17" s="7" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -2450,6 +2487,7 @@
         </is>
       </c>
       <c r="T18" s="5" t="inlineStr"/>
+      <c r="U18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -2510,6 +2548,7 @@
       <c r="R19" s="7" t="inlineStr"/>
       <c r="S19" s="7" t="inlineStr"/>
       <c r="T19" s="7" t="inlineStr"/>
+      <c r="U19" s="7" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -2570,6 +2609,7 @@
       <c r="R20" s="5" t="inlineStr"/>
       <c r="S20" s="5" t="inlineStr"/>
       <c r="T20" s="5" t="inlineStr"/>
+      <c r="U20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -2646,6 +2686,7 @@
         </is>
       </c>
       <c r="T21" s="7" t="inlineStr"/>
+      <c r="U21" s="7" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -2722,6 +2763,7 @@
         </is>
       </c>
       <c r="T22" s="5" t="inlineStr"/>
+      <c r="U22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -2802,6 +2844,7 @@
         </is>
       </c>
       <c r="T23" s="7" t="inlineStr"/>
+      <c r="U23" s="7" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -2862,6 +2905,7 @@
       <c r="R24" s="5" t="inlineStr"/>
       <c r="S24" s="5" t="inlineStr"/>
       <c r="T24" s="5" t="inlineStr"/>
+      <c r="U24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -2922,6 +2966,7 @@
       <c r="R25" s="7" t="inlineStr"/>
       <c r="S25" s="7" t="inlineStr"/>
       <c r="T25" s="7" t="inlineStr"/>
+      <c r="U25" s="7" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -2982,6 +3027,7 @@
       <c r="R26" s="5" t="inlineStr"/>
       <c r="S26" s="5" t="inlineStr"/>
       <c r="T26" s="5" t="inlineStr"/>
+      <c r="U26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -3042,9 +3088,10 @@
       <c r="R27" s="7" t="inlineStr"/>
       <c r="S27" s="7" t="inlineStr"/>
       <c r="T27" s="7" t="inlineStr"/>
+      <c r="U27" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T27"/>
+  <autoFilter ref="A1:U27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Align matching steps across workflows with Physical Altercation (WF-002) guide
Using WF-002 as the reference, standardize equivalent steps in the other
workflows:

- Parent Notification (WF-001/003/004/005 step 3, WF-001 step 2): email now sends
  AFTER the step (notifyOnStart false, notifyOnComplete true, notifyAssignee
  true, notifyApprovers false). WF-004 had no email; now matches.
- Disciplinary review/action (WF-003/004/005 step 4): send "Action Required" to
  the Safety Coordinator role, after the step (notifyOnStart false, notifyGroups
  Safety Coordinator, emailTemplate Action Required).

Driver-response, report-submission, and Documentation & Close steps already
matched (no email). Regenerated Incident-Tracker-Seed-Catalog.xlsx and refreshed
the README template note.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Incident-Tracker-Seed-Catalog.xlsx
+++ b/Incident-Tracker-Seed-Catalog.xlsx
@@ -646,7 +646,7 @@
     <row r="23">
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>• 'email_template' on a step references Email Templates.name. A blank means the step sends no templated email (though notify_* flags may still be set). Currently only WF-002 step 4 references a template ('Action Required'); the others are seeded as a reusable library.</t>
+          <t>• 'email_template' on a step references Email Templates.name. A blank means the step sends no templated email (though notify_* flags may still be set). The disciplinary-review steps (WF-002/003/004/005 step 4) reference the 'Action Required' template; the other templates are seeded as a reusable library.</t>
         </is>
       </c>
     </row>
@@ -1426,12 +1426,12 @@
       </c>
       <c r="Q3" s="7" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="R3" s="7" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="S3" s="7" t="inlineStr">
@@ -2046,12 +2046,12 @@
       <c r="O12" s="5" t="inlineStr"/>
       <c r="P12" s="5" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="Q12" s="5" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="R12" s="5" t="inlineStr">
@@ -2124,10 +2124,14 @@
       <c r="L13" s="7" t="inlineStr"/>
       <c r="M13" s="7" t="inlineStr"/>
       <c r="N13" s="7" t="inlineStr"/>
-      <c r="O13" s="7" t="inlineStr"/>
+      <c r="O13" s="7" t="inlineStr">
+        <is>
+          <t>Action Required</t>
+        </is>
+      </c>
       <c r="P13" s="7" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="Q13" s="7" t="inlineStr">
@@ -2145,7 +2149,11 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="T13" s="7" t="inlineStr"/>
+      <c r="T13" s="7" t="inlineStr">
+        <is>
+          <t>Safety Coordinator</t>
+        </is>
+      </c>
       <c r="U13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
@@ -2401,10 +2409,26 @@
       <c r="M17" s="7" t="inlineStr"/>
       <c r="N17" s="7" t="inlineStr"/>
       <c r="O17" s="7" t="inlineStr"/>
-      <c r="P17" s="7" t="inlineStr"/>
-      <c r="Q17" s="7" t="inlineStr"/>
-      <c r="R17" s="7" t="inlineStr"/>
-      <c r="S17" s="7" t="inlineStr"/>
+      <c r="P17" s="7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="Q17" s="7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="R17" s="7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="S17" s="7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
       <c r="T17" s="7" t="inlineStr"/>
       <c r="U17" s="7" t="inlineStr"/>
     </row>
@@ -2465,10 +2489,14 @@
       <c r="L18" s="5" t="inlineStr"/>
       <c r="M18" s="5" t="inlineStr"/>
       <c r="N18" s="5" t="inlineStr"/>
-      <c r="O18" s="5" t="inlineStr"/>
+      <c r="O18" s="5" t="inlineStr">
+        <is>
+          <t>Action Required</t>
+        </is>
+      </c>
       <c r="P18" s="5" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="Q18" s="5" t="inlineStr">
@@ -2486,7 +2514,11 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="T18" s="5" t="inlineStr"/>
+      <c r="T18" s="5" t="inlineStr">
+        <is>
+          <t>Safety Coordinator</t>
+        </is>
+      </c>
       <c r="U18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
@@ -2744,12 +2776,12 @@
       <c r="O22" s="5" t="inlineStr"/>
       <c r="P22" s="5" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="Q22" s="5" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="R22" s="5" t="inlineStr">
@@ -2822,10 +2854,14 @@
       <c r="L23" s="7" t="inlineStr"/>
       <c r="M23" s="7" t="inlineStr"/>
       <c r="N23" s="7" t="inlineStr"/>
-      <c r="O23" s="7" t="inlineStr"/>
+      <c r="O23" s="7" t="inlineStr">
+        <is>
+          <t>Action Required</t>
+        </is>
+      </c>
       <c r="P23" s="7" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="Q23" s="7" t="inlineStr">
@@ -2843,7 +2879,11 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="T23" s="7" t="inlineStr"/>
+      <c r="T23" s="7" t="inlineStr">
+        <is>
+          <t>Safety Coordinator</t>
+        </is>
+      </c>
       <c r="U23" s="7" t="inlineStr"/>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Safety Violation step 2: match Physical Altercation "Submit Incident Report"
Replace WF-005 step 2 ("Dispatch & Safety Coordinator Alert") with the same
details as WF-002 step 2: name "Submit Incident Report", driver submits via the
tablet app, 15 minutes, no email notification. Regenerated the seed catalog.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Incident-Tracker-Seed-Catalog.xlsx
+++ b/Incident-Tracker-Seed-Catalog.xlsx
@@ -2659,22 +2659,22 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Dispatch &amp; Safety Coordinator Alert</t>
+          <t>Submit Incident Report</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>For high-severity situations (emergency exit, wrong stop): notify dispatch and safety coordinator immediately</t>
+          <t>Driver submits the incident details — what occurred, injuries, and any threatening behavior — through the tablet app. Submitting the report notifies the safety coordinator.</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Safety Coordinator</t>
+          <t>Driver</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>10 minutes</t>
+          <t>15 minutes</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
@@ -2697,26 +2697,10 @@
       <c r="M21" s="7" t="inlineStr"/>
       <c r="N21" s="7" t="inlineStr"/>
       <c r="O21" s="7" t="inlineStr"/>
-      <c r="P21" s="7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="Q21" s="7" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="R21" s="7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="S21" s="7" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
+      <c r="P21" s="7" t="inlineStr"/>
+      <c r="Q21" s="7" t="inlineStr"/>
+      <c r="R21" s="7" t="inlineStr"/>
+      <c r="S21" s="7" t="inlineStr"/>
       <c r="T21" s="7" t="inlineStr"/>
       <c r="U21" s="7" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Safety Violation step 4: match Physical Altercation "Disciplinary Action Review"
Make WF-005 step 4 identical to WF-002 step 4: rename to "Disciplinary Action
Review", use its description, 1 hour duration, and required = true. Role,
approval, and the Action Required -> Safety Coordinator email already matched.
Regenerated the seed catalog.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Incident-Tracker-Seed-Catalog.xlsx
+++ b/Incident-Tracker-Seed-Catalog.xlsx
@@ -2797,12 +2797,12 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Safety Review &amp; Disciplinary Action</t>
+          <t>Disciplinary Action Review</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>Review incident severity and history. Determine if disciplinary measures are warranted.</t>
+          <t>Administrator reviews incident and determines appropriate disciplinary measures</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
@@ -2812,12 +2812,12 @@
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>20 minutes</t>
+          <t>1 hour</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I23" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Property Damage step 2: send Action Required to Safety Coordinator
Fleet Manager Review now sends the "Action Required" email template to the
Safety Coordinator role (notifyGroups: Safety Coordinator, emailTemplate: Action
Required). Existing send timing (on start + on complete) preserved. Regenerated
the seed catalog and updated the README template note.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Incident-Tracker-Seed-Catalog.xlsx
+++ b/Incident-Tracker-Seed-Catalog.xlsx
@@ -646,7 +646,7 @@
     <row r="23">
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>• 'email_template' on a step references Email Templates.name. A blank means the step sends no templated email (though notify_* flags may still be set). The disciplinary-review steps (WF-002/003/004/005 step 4) reference the 'Action Required' template; the other templates are seeded as a reusable library.</t>
+          <t>• 'email_template' on a step references Email Templates.name. A blank means the step sends no templated email (though notify_* flags may still be set). The disciplinary-review steps (WF-002/003/004/005 step 4) and WF-004 step 2 (Fleet Manager Review) reference the 'Action Required' template; the other templates are seeded as a reusable library.</t>
         </is>
       </c>
     </row>
@@ -2331,7 +2331,11 @@
       <c r="L16" s="5" t="inlineStr"/>
       <c r="M16" s="5" t="inlineStr"/>
       <c r="N16" s="5" t="inlineStr"/>
-      <c r="O16" s="5" t="inlineStr"/>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>Action Required</t>
+        </is>
+      </c>
       <c r="P16" s="5" t="inlineStr">
         <is>
           <t>TRUE</t>
@@ -2352,7 +2356,11 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="T16" s="5" t="inlineStr"/>
+      <c r="T16" s="5" t="inlineStr">
+        <is>
+          <t>Safety Coordinator</t>
+        </is>
+      </c>
       <c r="U16" s="5" t="inlineStr"/>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
Property Damage: Repair Scheduling email + new coordinator close step
- Step 5 (Repair Scheduling) now sends the "Action Required" email to the
  Safety Coordinator after the step completes.
- Add step 6 "Documentation & Close" (Safety Coordinator) so the coordinator
  closes the incident at the end of the workflow.

Updated workflows.ts and the generator; regenerated Incident-Tracker-Seed-Catalog.xlsx
(now 27 workflow steps) and refreshed the README template note.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Incident-Tracker-Seed-Catalog.xlsx
+++ b/Incident-Tracker-Seed-Catalog.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Incident Types'!$A$1:$F$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Workflows'!$A$1:$E$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Workflow Steps'!$A$1:$U$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Workflow Steps'!$A$1:$U$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Step Templates'!$A$1:$K$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Email Templates'!$A$1:$H$4</definedName>
   </definedNames>
@@ -646,7 +646,7 @@
     <row r="23">
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>• 'email_template' on a step references Email Templates.name. A blank means the step sends no templated email (though notify_* flags may still be set). The disciplinary-review steps (WF-002/003/004/005 step 4) and WF-004 step 2 (Fleet Manager Review) reference the 'Action Required' template; the other templates are seeded as a reusable library.</t>
+          <t>• 'email_template' on a step references Email Templates.name. A blank means the step sends no templated email (though notify_* flags may still be set). Several steps reference the 'Action Required' template — the disciplinary-review step 4s (WF-002/003/004/005) and WF-004 steps 2 and 5; the other templates are seeded as a reusable library.</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U27"/>
+  <dimension ref="A1:U28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2582,46 +2582,70 @@
       <c r="L19" s="7" t="inlineStr"/>
       <c r="M19" s="7" t="inlineStr"/>
       <c r="N19" s="7" t="inlineStr"/>
-      <c r="O19" s="7" t="inlineStr"/>
-      <c r="P19" s="7" t="inlineStr"/>
-      <c r="Q19" s="7" t="inlineStr"/>
-      <c r="R19" s="7" t="inlineStr"/>
-      <c r="S19" s="7" t="inlineStr"/>
-      <c r="T19" s="7" t="inlineStr"/>
+      <c r="O19" s="7" t="inlineStr">
+        <is>
+          <t>Action Required</t>
+        </is>
+      </c>
+      <c r="P19" s="7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="Q19" s="7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="R19" s="7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="S19" s="7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="T19" s="7" t="inlineStr">
+        <is>
+          <t>Safety Coordinator</t>
+        </is>
+      </c>
       <c r="U19" s="7" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>WF-005</t>
+          <t>WF-004</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>step-1</t>
+          <t>step-6</t>
         </is>
       </c>
       <c r="C20" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Immediate Safety Response</t>
+          <t>Documentation &amp; Close</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Driver addresses the safety issue, secures the situation, and documents the incident</t>
+          <t>Complete incident documentation and close case</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Driver</t>
+          <t>Safety Coordinator</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>15 minutes</t>
+          <t>20 minutes</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
@@ -2659,20 +2683,20 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>step-2</t>
+          <t>step-1</t>
         </is>
       </c>
       <c r="C21" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Submit Incident Report</t>
+          <t>Immediate Safety Response</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Driver submits the incident details — what occurred, injuries, and any threatening behavior — through the tablet app. Submitting the report notifies the safety coordinator.</t>
+          <t>Driver addresses the safety issue, secures the situation, and documents the incident</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
@@ -2720,25 +2744,25 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>step-3</t>
+          <t>step-2</t>
         </is>
       </c>
       <c r="C22" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Parent Notification</t>
+          <t>Submit Incident Report</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Contact parent/guardian to inform them of the safety violation and reinforce bus safety expectations</t>
+          <t>Driver submits the incident details — what occurred, injuries, and any threatening behavior — through the tablet app. Submitting the report notifies the safety coordinator.</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Safety Coordinator</t>
+          <t>Driver</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -2766,26 +2790,10 @@
       <c r="M22" s="5" t="inlineStr"/>
       <c r="N22" s="5" t="inlineStr"/>
       <c r="O22" s="5" t="inlineStr"/>
-      <c r="P22" s="5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="Q22" s="5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="R22" s="5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="S22" s="5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
+      <c r="P22" s="5" t="inlineStr"/>
+      <c r="Q22" s="5" t="inlineStr"/>
+      <c r="R22" s="5" t="inlineStr"/>
+      <c r="S22" s="5" t="inlineStr"/>
       <c r="T22" s="5" t="inlineStr"/>
       <c r="U22" s="5" t="inlineStr"/>
     </row>
@@ -2797,30 +2805,30 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>step-4</t>
+          <t>step-3</t>
         </is>
       </c>
       <c r="C23" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Disciplinary Action Review</t>
+          <t>Parent Notification</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>Administrator reviews incident and determines appropriate disciplinary measures</t>
+          <t>Contact parent/guardian to inform them of the safety violation and reinforce bus safety expectations</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Safety Coordinator</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>1 hour</t>
+          <t>15 minutes</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
@@ -2830,14 +2838,10 @@
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="J23" s="7" t="inlineStr">
-        <is>
-          <t>Administrator</t>
-        </is>
-      </c>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J23" s="7" t="inlineStr"/>
       <c r="K23" s="7" t="inlineStr">
         <is>
           <t>manual</t>
@@ -2846,11 +2850,7 @@
       <c r="L23" s="7" t="inlineStr"/>
       <c r="M23" s="7" t="inlineStr"/>
       <c r="N23" s="7" t="inlineStr"/>
-      <c r="O23" s="7" t="inlineStr">
-        <is>
-          <t>Action Required</t>
-        </is>
-      </c>
+      <c r="O23" s="7" t="inlineStr"/>
       <c r="P23" s="7" t="inlineStr">
         <is>
           <t>FALSE</t>
@@ -2868,14 +2868,10 @@
       </c>
       <c r="S23" s="7" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T23" s="7" t="inlineStr">
-        <is>
-          <t>Safety Coordinator</t>
-        </is>
-      </c>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="T23" s="7" t="inlineStr"/>
       <c r="U23" s="7" t="inlineStr"/>
     </row>
     <row r="24">
@@ -2886,30 +2882,30 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>step-5</t>
+          <t>step-4</t>
         </is>
       </c>
       <c r="C24" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Documentation &amp; Close</t>
+          <t>Disciplinary Action Review</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Complete all documentation and close the incident</t>
+          <t>Administrator reviews incident and determines appropriate disciplinary measures</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Safety Coordinator</t>
+          <t>Administrator</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>10 minutes</t>
+          <t>1 hour</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
@@ -2919,10 +2915,14 @@
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="J24" s="5" t="inlineStr"/>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>Administrator</t>
+        </is>
+      </c>
       <c r="K24" s="5" t="inlineStr">
         <is>
           <t>manual</t>
@@ -2931,41 +2931,65 @@
       <c r="L24" s="5" t="inlineStr"/>
       <c r="M24" s="5" t="inlineStr"/>
       <c r="N24" s="5" t="inlineStr"/>
-      <c r="O24" s="5" t="inlineStr"/>
-      <c r="P24" s="5" t="inlineStr"/>
-      <c r="Q24" s="5" t="inlineStr"/>
-      <c r="R24" s="5" t="inlineStr"/>
-      <c r="S24" s="5" t="inlineStr"/>
-      <c r="T24" s="5" t="inlineStr"/>
+      <c r="O24" s="5" t="inlineStr">
+        <is>
+          <t>Action Required</t>
+        </is>
+      </c>
+      <c r="P24" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="Q24" s="5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="R24" s="5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="S24" s="5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T24" s="5" t="inlineStr">
+        <is>
+          <t>Safety Coordinator</t>
+        </is>
+      </c>
       <c r="U24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>WF-006</t>
+          <t>WF-005</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>step-1</t>
+          <t>step-5</t>
         </is>
       </c>
       <c r="C25" s="7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Record Witness Statement</t>
+          <t>Documentation &amp; Close</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>Driver or staff records the witness/bystander account of what they saw or how they helped. No fault is assigned to this student.</t>
+          <t>Complete all documentation and close the incident</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>Driver</t>
+          <t>Safety Coordinator</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -3008,25 +3032,25 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>step-2</t>
+          <t>step-1</t>
         </is>
       </c>
       <c r="C26" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Link to Related Incident</t>
+          <t>Record Witness Statement</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Safety coordinator reviews the statement and links it to the related disciplinary incident (e.g. the physical altercation) for context.</t>
+          <t>Driver or staff records the witness/bystander account of what they saw or how they helped. No fault is assigned to this student.</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Safety Coordinator</t>
+          <t>Driver</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -3036,7 +3060,7 @@
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
@@ -3069,20 +3093,20 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>step-3</t>
+          <t>step-2</t>
         </is>
       </c>
       <c r="C27" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>File &amp; Close</t>
+          <t>Link to Related Incident</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>File the witness statement and close. No disciplinary measures or parent notification are required for the witness.</t>
+          <t>Safety coordinator reviews the statement and links it to the related disciplinary incident (e.g. the physical altercation) for context.</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
@@ -3092,12 +3116,12 @@
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>5 minutes</t>
+          <t>10 minutes</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="I27" s="7" t="inlineStr">
@@ -3122,8 +3146,69 @@
       <c r="T27" s="7" t="inlineStr"/>
       <c r="U27" s="7" t="inlineStr"/>
     </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>WF-006</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>step-3</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>File &amp; Close</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>File the witness statement and close. No disciplinary measures or parent notification are required for the witness.</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Safety Coordinator</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>5 minutes</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr"/>
+      <c r="K28" s="5" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="L28" s="5" t="inlineStr"/>
+      <c r="M28" s="5" t="inlineStr"/>
+      <c r="N28" s="5" t="inlineStr"/>
+      <c r="O28" s="5" t="inlineStr"/>
+      <c r="P28" s="5" t="inlineStr"/>
+      <c r="Q28" s="5" t="inlineStr"/>
+      <c r="R28" s="5" t="inlineStr"/>
+      <c r="S28" s="5" t="inlineStr"/>
+      <c r="T28" s="5" t="inlineStr"/>
+      <c r="U28" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U27"/>
+  <autoFilter ref="A1:U28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Prohibited Items step 2: match Physical Altercation "Submit Incident Report"
Replace WF-003 step 2 ("Safety Coordinator & Administration Alert") with the
same details as WF-002 step 2: "Submit Incident Report", driver submits via the
tablet app, 15 minutes, no email notification. Regenerated the seed catalog.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Incident-Tracker-Seed-Catalog.xlsx
+++ b/Incident-Tracker-Seed-Catalog.xlsx
@@ -1929,12 +1929,12 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Safety Coordinator &amp; Administration Alert</t>
+          <t>Submit Incident Report</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Notify safety coordinator and school administration; for illegal substances or weapons, notify law enforcement</t>
+          <t>Driver submits the incident details — what occurred, injuries, and any threatening behavior — through the tablet app. Submitting the report notifies the safety coordinator.</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -1967,26 +1967,10 @@
       <c r="M11" s="7" t="inlineStr"/>
       <c r="N11" s="7" t="inlineStr"/>
       <c r="O11" s="7" t="inlineStr"/>
-      <c r="P11" s="7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="Q11" s="7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="R11" s="7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="S11" s="7" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
+      <c r="P11" s="7" t="inlineStr"/>
+      <c r="Q11" s="7" t="inlineStr"/>
+      <c r="R11" s="7" t="inlineStr"/>
+      <c r="S11" s="7" t="inlineStr"/>
       <c r="T11" s="7" t="inlineStr"/>
       <c r="U11" s="7" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Witness / Bystander workflow: single non-required step
Remove steps 2 (Link to Related Incident) and 3 (File & Close) from WF-006. The
linking/filing happens automatically when the driver captures the incident; the
remaining step exists only to assign the witness statement to the student. Make
the lone Record Witness Statement step not required, with no email notification.
Regenerated the seed catalog (now 25 workflow steps).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Incident-Tracker-Seed-Catalog.xlsx
+++ b/Incident-Tracker-Seed-Catalog.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Incident Types'!$A$1:$F$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Workflows'!$A$1:$E$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Workflow Steps'!$A$1:$U$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Workflow Steps'!$A$1:$U$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Step Templates'!$A$1:$K$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Email Templates'!$A$1:$H$4</definedName>
   </definedNames>
@@ -1171,7 +1171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U28"/>
+  <dimension ref="A1:U26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3044,7 +3044,7 @@
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
@@ -3069,130 +3069,8 @@
       <c r="T26" s="5" t="inlineStr"/>
       <c r="U26" s="5" t="inlineStr"/>
     </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>WF-006</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>step-2</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>Link to Related Incident</t>
-        </is>
-      </c>
-      <c r="E27" s="8" t="inlineStr">
-        <is>
-          <t>Safety coordinator reviews the statement and links it to the related disciplinary incident (e.g. the physical altercation) for context.</t>
-        </is>
-      </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>Safety Coordinator</t>
-        </is>
-      </c>
-      <c r="G27" s="7" t="inlineStr">
-        <is>
-          <t>10 minutes</t>
-        </is>
-      </c>
-      <c r="H27" s="7" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="I27" s="7" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="J27" s="7" t="inlineStr"/>
-      <c r="K27" s="7" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-      <c r="L27" s="7" t="inlineStr"/>
-      <c r="M27" s="7" t="inlineStr"/>
-      <c r="N27" s="7" t="inlineStr"/>
-      <c r="O27" s="7" t="inlineStr"/>
-      <c r="P27" s="7" t="inlineStr"/>
-      <c r="Q27" s="7" t="inlineStr"/>
-      <c r="R27" s="7" t="inlineStr"/>
-      <c r="S27" s="7" t="inlineStr"/>
-      <c r="T27" s="7" t="inlineStr"/>
-      <c r="U27" s="7" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>WF-006</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>step-3</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>File &amp; Close</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>File the witness statement and close. No disciplinary measures or parent notification are required for the witness.</t>
-        </is>
-      </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>Safety Coordinator</t>
-        </is>
-      </c>
-      <c r="G28" s="5" t="inlineStr">
-        <is>
-          <t>5 minutes</t>
-        </is>
-      </c>
-      <c r="H28" s="5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="I28" s="5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="J28" s="5" t="inlineStr"/>
-      <c r="K28" s="5" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-      <c r="L28" s="5" t="inlineStr"/>
-      <c r="M28" s="5" t="inlineStr"/>
-      <c r="N28" s="5" t="inlineStr"/>
-      <c r="O28" s="5" t="inlineStr"/>
-      <c r="P28" s="5" t="inlineStr"/>
-      <c r="Q28" s="5" t="inlineStr"/>
-      <c r="R28" s="5" t="inlineStr"/>
-      <c r="S28" s="5" t="inlineStr"/>
-      <c r="T28" s="5" t="inlineStr"/>
-      <c r="U28" s="5" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:U28"/>
+  <autoFilter ref="A1:U26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Step template library: remove Safety Coordinator Alert, Admin Notification, Fleet/Repair
Delete the comm-safety-alert, comm-admin-notify, and admin-fleet-repair step
templates from the library (and their seed-catalog entries). Library now has 5
templates: Parent/Guardian Notification, Photo & Evidence Documentation,
Disciplinary Review, Law Enforcement Contact, Documentation & Close.
Regenerated Incident-Tracker-Seed-Catalog.xlsx.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Incident-Tracker-Seed-Catalog.xlsx
+++ b/Incident-Tracker-Seed-Catalog.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Incident Types'!$A$1:$F$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Workflows'!$A$1:$E$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Workflow Steps'!$A$1:$U$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Step Templates'!$A$1:$N$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Step Templates'!$A$1:$N$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Email Templates'!$A$1:$H$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3081,7 +3081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3235,32 +3235,32 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>comm-safety-alert</t>
+          <t>doc-photo-evidence</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Safety Coordinator Alert</t>
+          <t>Photo &amp; Evidence Documentation</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Notification</t>
+          <t>Review &amp; Action</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>Send urgent notification to safety coordinator with full incident details</t>
+          <t>Photograph damage or relevant scene, document physical evidence</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>Safety Coordinator</t>
+          <t>Driver</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>15 minutes</t>
+          <t>20 minutes</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
@@ -3268,74 +3268,62 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="I3" s="7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="J3" s="7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+      <c r="H3" s="7" t="inlineStr"/>
+      <c r="I3" s="7" t="inlineStr"/>
+      <c r="J3" s="7" t="inlineStr"/>
       <c r="K3" s="7" t="inlineStr"/>
       <c r="L3" s="7" t="inlineStr"/>
       <c r="M3" s="7" t="inlineStr"/>
       <c r="N3" s="7" t="inlineStr">
         <is>
-          <t>safety, coordinator, alert, urgent</t>
+          <t>photo, evidence, documentation, damage</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>comm-admin-notify</t>
+          <t>admin-disciplinary-review</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Administrator / Principal Notification</t>
+          <t>Disciplinary Review</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Notification</t>
+          <t>Review &amp; Action</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>Notify school administrator or principal of the incident</t>
+          <t>Administrator reviews incident and determines appropriate disciplinary action; requires approval before proceeding</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>School Principal</t>
+          <t>Administrator</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>20 minutes</t>
+          <t>1 hour</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
@@ -3343,24 +3331,36 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr"/>
-      <c r="L4" s="5" t="inlineStr"/>
-      <c r="M4" s="5" t="inlineStr"/>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>Safety Coordinator</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>Action Required</t>
+        </is>
+      </c>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>administrator, principal, school, notification</t>
+          <t>disciplinary, review, administrator, approval</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>doc-photo-evidence</t>
+          <t>admin-police-report</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Photo &amp; Evidence Documentation</t>
+          <t>Law Enforcement Contact</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -3370,290 +3370,98 @@
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>Photograph damage or relevant scene, document physical evidence</t>
+          <t>File police report or coordinate with law enforcement for criminal incidents</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Driver</t>
+          <t>Administrator</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>20 minutes</t>
+          <t>1 hour</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr"/>
-      <c r="I5" s="7" t="inlineStr"/>
-      <c r="J5" s="7" t="inlineStr"/>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
       <c r="K5" s="7" t="inlineStr"/>
       <c r="L5" s="7" t="inlineStr"/>
       <c r="M5" s="7" t="inlineStr"/>
       <c r="N5" s="7" t="inlineStr">
         <is>
-          <t>photo, evidence, documentation, damage</t>
+          <t>police, law enforcement, criminal, report</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>admin-disciplinary-review</t>
+          <t>follow-close-incident</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Disciplinary Review</t>
+          <t>Documentation &amp; Close</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Review &amp; Action</t>
+          <t>Close Out</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Administrator reviews incident and determines appropriate disciplinary action; requires approval before proceeding</t>
+          <t>Complete all incident documentation, finalize the record, and close the case</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Safety Coordinator</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>1 hour</t>
+          <t>15 minutes</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="K6" s="5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="L6" s="5" t="inlineStr">
-        <is>
-          <t>Safety Coordinator</t>
-        </is>
-      </c>
-      <c r="M6" s="5" t="inlineStr">
-        <is>
-          <t>Action Required</t>
-        </is>
-      </c>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr"/>
+      <c r="I6" s="5" t="inlineStr"/>
+      <c r="J6" s="5" t="inlineStr"/>
+      <c r="K6" s="5" t="inlineStr"/>
+      <c r="L6" s="5" t="inlineStr"/>
+      <c r="M6" s="5" t="inlineStr"/>
       <c r="N6" s="5" t="inlineStr">
         <is>
-          <t>disciplinary, review, administrator, approval</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>admin-police-report</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Law Enforcement Contact</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Review &amp; Action</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>File police report or coordinate with law enforcement for criminal incidents</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>Administrator</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>1 hour</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="I7" s="7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="J7" s="7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="K7" s="7" t="inlineStr"/>
-      <c r="L7" s="7" t="inlineStr"/>
-      <c r="M7" s="7" t="inlineStr"/>
-      <c r="N7" s="7" t="inlineStr">
-        <is>
-          <t>police, law enforcement, criminal, report</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>admin-fleet-repair</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Fleet / Repair Coordination</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Review &amp; Action</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>Fleet manager assesses damage, provides repair estimate, and schedules vehicle repairs</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Fleet Manager</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>2 hours</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="J8" s="5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="K8" s="5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="L8" s="5" t="inlineStr">
-        <is>
-          <t>Safety Coordinator</t>
-        </is>
-      </c>
-      <c r="M8" s="5" t="inlineStr">
-        <is>
-          <t>Action Required</t>
-        </is>
-      </c>
-      <c r="N8" s="5" t="inlineStr">
-        <is>
-          <t>fleet, repair, vehicle, damage, maintenance</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>follow-close-incident</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Documentation &amp; Close</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>Close Out</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>Complete all incident documentation, finalize the record, and close the case</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>Safety Coordinator</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>15 minutes</t>
-        </is>
-      </c>
-      <c r="G9" s="7" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="H9" s="7" t="inlineStr"/>
-      <c r="I9" s="7" t="inlineStr"/>
-      <c r="J9" s="7" t="inlineStr"/>
-      <c r="K9" s="7" t="inlineStr"/>
-      <c r="L9" s="7" t="inlineStr"/>
-      <c r="M9" s="7" t="inlineStr"/>
-      <c r="N9" s="7" t="inlineStr">
-        <is>
           <t>close, documentation, finalize, complete</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N9"/>
+  <autoFilter ref="A1:N6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Law Enforcement Contact template: no email notifications
Remove the emailNotifications from the admin-police-report step template so it
sends no email. Regenerated the seed catalog.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Incident-Tracker-Seed-Catalog.xlsx
+++ b/Incident-Tracker-Seed-Catalog.xlsx
@@ -3388,21 +3388,9 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="I5" s="7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="J5" s="7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+      <c r="H5" s="7" t="inlineStr"/>
+      <c r="I5" s="7" t="inlineStr"/>
+      <c r="J5" s="7" t="inlineStr"/>
       <c r="K5" s="7" t="inlineStr"/>
       <c r="L5" s="7" t="inlineStr"/>
       <c r="M5" s="7" t="inlineStr"/>

</xml_diff>